<commit_message>
latest dark UI with updated changes
</commit_message>
<xml_diff>
--- a/reports/aws_pricing_forecast.xlsx
+++ b/reports/aws_pricing_forecast.xlsx
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -740,14 +740,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AWS 5-Year Cost Forecast  |  PNB  |  24 Mar 2026  |  Inflation: 4.0%/yr</t>
+          <t>AWS 5-Year Cost Forecast  |  PAYTM  |  09 Apr 2026  |  Inflation: 4.0%/yr</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Base Monthly: $10,158.41  |  Annual Y1: $121,900.92  |  3-Year: $365,702.76</t>
+          <t>Base Monthly: $6,147.27  |  Annual Y1: $73,767.24  |  3-Year: $221,301.72</t>
         </is>
       </c>
     </row>
@@ -978,25 +978,25 @@
         </is>
       </c>
       <c r="D10" s="12" t="n">
-        <v>41.45</v>
+        <v>32.45</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>497.4</v>
+        <v>389.4</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>517.3</v>
+        <v>404.98</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>537.99</v>
+        <v>421.18</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>559.51</v>
+        <v>438.02</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>581.89</v>
+        <v>455.54</v>
       </c>
       <c r="J10" s="12" t="n">
-        <v>2694.09</v>
+        <v>2109.12</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -1099,25 +1099,25 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>3486.72</v>
+        <v>1162.24</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>41840.64</v>
+        <v>13946.88</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>43514.27</v>
+        <v>14504.76</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>45254.84</v>
+        <v>15084.95</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>47065.03</v>
+        <v>15688.34</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>48947.63</v>
+        <v>16315.88</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>226622.41</v>
+        <v>75540.81</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -1133,719 +1133,681 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>m5.2xlarge</t>
+          <t>m5.4xlarge</t>
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>321.28</v>
+        <v>601.6</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>3855.36</v>
+        <v>7219.2</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>4009.57</v>
+        <v>7507.97</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>4169.96</v>
+        <v>7808.29</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>4336.76</v>
+        <v>8120.62</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>4510.23</v>
+        <v>8445.440000000001</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>20881.88</v>
+        <v>39101.52</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Kubernetes Cluster</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Worker Nodes Linux/RHEL for EFK - optional</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>m5.2xlarge</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="n">
-        <v>724.48</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>8693.76</v>
-      </c>
-      <c r="F16" s="9" t="n">
-        <v>9041.51</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>9403.17</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>9779.299999999999</v>
-      </c>
-      <c r="I16" s="9" t="n">
-        <v>10170.47</v>
-      </c>
-      <c r="J16" s="9" t="n">
-        <v>47088.21</v>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Cloud Managed K8s</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>EKS</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>73</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>876</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>911.04</v>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>947.48</v>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>985.38</v>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>1024.8</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>4744.7</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>CloudWatch Monitoring</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>CloudWatch</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>708</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>736.3200000000001</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>765.77</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>796.4</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>828.26</v>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>3834.75</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PGSQL Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>PGSQL Database</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Linux Nodes – Database server (Primary)</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>r5.8xlarge</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>2991.36</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>35896.32</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>37332.17</v>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>38825.46</v>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>40378.48</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>41993.62</v>
+      </c>
+      <c r="J20" s="12" t="n">
+        <v>194426.05</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>PGSQL Database</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Nodes – Cluster (etcd+haproxy, pgbackrest)</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>r5.large</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>399.92</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>4799.04</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>4991</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>5190.64</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>5398.27</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>5614.2</v>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>25993.15</v>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>PGSQL Database</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Storage: SAN (Primary PostgreSQL DB)</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>EBS io2</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>312</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>324.48</v>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>337.46</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>350.96</v>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>1624.9</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>S3 Storage + Replication</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>EBS io2</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>300</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>312</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>324.48</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>337.46</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>350.96</v>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>1624.9</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Category Subtotals</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Caching &amp; Session</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>All services</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>481.8</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>5781.6</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>6012.86</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>6253.38</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>6503.51</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>6763.65</v>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>31315</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Infrastructure &amp; Monitoring</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>All services</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>328.35</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>3940.2</v>
+      </c>
+      <c r="F28" s="12" t="n">
+        <v>4097.81</v>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>4261.72</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>4432.19</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>4609.48</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>21341.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Kubernetes Cluster</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Cloud Managed K8s</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>EKS</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>73</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>876</v>
-      </c>
-      <c r="F17" s="12" t="n">
-        <v>911.04</v>
-      </c>
-      <c r="G17" s="12" t="n">
-        <v>947.48</v>
-      </c>
-      <c r="H17" s="12" t="n">
-        <v>985.38</v>
-      </c>
-      <c r="I17" s="12" t="n">
-        <v>1024.8</v>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>4744.7</v>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Operations</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>All services</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>1836.84</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>22042.08</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>22923.76</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>23840.71</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>24794.34</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>25786.12</v>
+      </c>
+      <c r="J29" s="9" t="n">
+        <v>119387.01</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>CloudWatch Monitoring</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>CloudWatch</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="n">
-        <v>80</v>
-      </c>
-      <c r="E19" s="9" t="n">
-        <v>960</v>
-      </c>
-      <c r="F19" s="9" t="n">
-        <v>998.4</v>
-      </c>
-      <c r="G19" s="9" t="n">
-        <v>1038.34</v>
-      </c>
-      <c r="H19" s="9" t="n">
-        <v>1079.87</v>
-      </c>
-      <c r="I19" s="9" t="n">
-        <v>1123.06</v>
-      </c>
-      <c r="J19" s="9" t="n">
-        <v>5199.67</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PGSQL Database</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>All services</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="E30" s="12" t="n">
+        <v>708</v>
+      </c>
+      <c r="F30" s="12" t="n">
+        <v>736.3200000000001</v>
+      </c>
+      <c r="G30" s="12" t="n">
+        <v>765.77</v>
+      </c>
+      <c r="H30" s="12" t="n">
+        <v>796.4</v>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>828.26</v>
+      </c>
+      <c r="J30" s="12" t="n">
+        <v>3834.75</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>PGSQL Database</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Linux Nodes – Database server (Primary)</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>r5.8xlarge</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="n">
-        <v>2991.36</v>
-      </c>
-      <c r="E21" s="12" t="n">
-        <v>35896.32</v>
-      </c>
-      <c r="F21" s="12" t="n">
-        <v>37332.17</v>
-      </c>
-      <c r="G21" s="12" t="n">
-        <v>38825.46</v>
-      </c>
-      <c r="H21" s="12" t="n">
-        <v>40378.48</v>
-      </c>
-      <c r="I21" s="12" t="n">
-        <v>41993.62</v>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>194426.05</v>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>PGSQL Database</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Linux Nodes – Cluster (etcd+haproxy, pgbackrest)</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>r5.large</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="n">
-        <v>399.92</v>
-      </c>
-      <c r="E22" s="9" t="n">
-        <v>4799.04</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>4991</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>5190.64</v>
-      </c>
-      <c r="H22" s="9" t="n">
-        <v>5398.27</v>
-      </c>
-      <c r="I22" s="9" t="n">
-        <v>5614.2</v>
-      </c>
-      <c r="J22" s="9" t="n">
-        <v>25993.15</v>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>PGSQL Database</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Storage: SAN (Primary DB)</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>EBS io2</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>525</v>
-      </c>
-      <c r="E23" s="12" t="n">
-        <v>6300</v>
-      </c>
-      <c r="F23" s="12" t="n">
-        <v>6552</v>
-      </c>
-      <c r="G23" s="12" t="n">
-        <v>6814.08</v>
-      </c>
-      <c r="H23" s="12" t="n">
-        <v>7086.64</v>
-      </c>
-      <c r="I23" s="12" t="n">
-        <v>7370.11</v>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>34122.83</v>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  S3</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>All services</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>3416.28</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>40995.36</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>42635.17</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>44340.58</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>46114.2</v>
+      </c>
+      <c r="I31" s="9" t="n">
+        <v>47958.77</v>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>222044.08</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>S3 Storage + Replication</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>EBS io2</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="n">
-        <v>737.5</v>
-      </c>
-      <c r="E25" s="9" t="n">
-        <v>8850</v>
-      </c>
-      <c r="F25" s="9" t="n">
-        <v>9204</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>9572.16</v>
-      </c>
-      <c r="H25" s="9" t="n">
-        <v>9955.049999999999</v>
-      </c>
-      <c r="I25" s="9" t="n">
-        <v>10353.25</v>
-      </c>
-      <c r="J25" s="9" t="n">
-        <v>47934.46</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Category Subtotals</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Caching &amp; Session</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>All services</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D28" s="9" t="n">
-        <v>481.8</v>
-      </c>
-      <c r="E28" s="9" t="n">
-        <v>5781.6</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <v>6012.86</v>
-      </c>
-      <c r="G28" s="9" t="n">
-        <v>6253.38</v>
-      </c>
-      <c r="H28" s="9" t="n">
-        <v>6503.51</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <v>6763.65</v>
-      </c>
-      <c r="J28" s="9" t="n">
-        <v>31315</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>Infrastructure &amp; Monitoring</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="D32" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="E32" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="F32" s="12" t="n">
+        <v>312</v>
+      </c>
+      <c r="G32" s="12" t="n">
+        <v>324.48</v>
+      </c>
+      <c r="H32" s="12" t="n">
+        <v>337.46</v>
+      </c>
+      <c r="I32" s="12" t="n">
+        <v>350.96</v>
+      </c>
+      <c r="J32" s="12" t="n">
+        <v>1624.9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Security &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>All services</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D29" s="12" t="n">
-        <v>337.35</v>
-      </c>
-      <c r="E29" s="12" t="n">
-        <v>4048.2</v>
-      </c>
-      <c r="F29" s="12" t="n">
-        <v>4210.13</v>
-      </c>
-      <c r="G29" s="12" t="n">
-        <v>4378.53</v>
-      </c>
-      <c r="H29" s="12" t="n">
-        <v>4553.67</v>
-      </c>
-      <c r="I29" s="12" t="n">
-        <v>4735.82</v>
-      </c>
-      <c r="J29" s="12" t="n">
-        <v>21926.35</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Kubernetes Cluster</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>All services</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="n">
-        <v>4605.48</v>
-      </c>
-      <c r="E30" s="9" t="n">
-        <v>55265.76</v>
-      </c>
-      <c r="F30" s="9" t="n">
-        <v>57476.39</v>
-      </c>
-      <c r="G30" s="9" t="n">
-        <v>59775.45</v>
-      </c>
-      <c r="H30" s="9" t="n">
-        <v>62166.46</v>
-      </c>
-      <c r="I30" s="9" t="n">
-        <v>64653.12</v>
-      </c>
-      <c r="J30" s="9" t="n">
-        <v>299337.18</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>All services</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="E31" s="12" t="n">
-        <v>960</v>
-      </c>
-      <c r="F31" s="12" t="n">
-        <v>998.4</v>
-      </c>
-      <c r="G31" s="12" t="n">
-        <v>1038.34</v>
-      </c>
-      <c r="H31" s="12" t="n">
-        <v>1079.87</v>
-      </c>
-      <c r="I31" s="12" t="n">
-        <v>1123.06</v>
-      </c>
-      <c r="J31" s="12" t="n">
-        <v>5199.67</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>PGSQL Database</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>All services</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="n">
-        <v>3916.28</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <v>46995.36</v>
-      </c>
-      <c r="F32" s="9" t="n">
-        <v>48875.17</v>
-      </c>
-      <c r="G32" s="9" t="n">
-        <v>50830.18</v>
-      </c>
-      <c r="H32" s="9" t="n">
-        <v>52863.39</v>
-      </c>
-      <c r="I32" s="9" t="n">
-        <v>54977.92</v>
-      </c>
-      <c r="J32" s="9" t="n">
-        <v>254542.02</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>S3</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>All services</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D33" s="12" t="n">
-        <v>737.5</v>
-      </c>
-      <c r="E33" s="12" t="n">
-        <v>8850</v>
-      </c>
-      <c r="F33" s="12" t="n">
-        <v>9204</v>
-      </c>
-      <c r="G33" s="12" t="n">
-        <v>9572.16</v>
-      </c>
-      <c r="H33" s="12" t="n">
-        <v>9955.049999999999</v>
-      </c>
-      <c r="I33" s="12" t="n">
-        <v>10353.25</v>
-      </c>
-      <c r="J33" s="12" t="n">
-        <v>47934.46</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>Security &amp; Compliance</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>All services</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="n">
+      <c r="D33" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="9" t="n">
+      <c r="E33" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="9" t="n">
+      <c r="F33" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="9" t="n">
+      <c r="G33" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="9" t="n">
+      <c r="H33" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="I34" s="9" t="n">
+      <c r="I33" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="J34" s="9" t="n">
+      <c r="J33" s="9" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr"/>
-      <c r="C35" s="15" t="inlineStr"/>
-      <c r="D35" s="16" t="n">
-        <v>10158.41</v>
-      </c>
-      <c r="E35" s="16" t="n">
-        <v>121900.92</v>
-      </c>
-      <c r="F35" s="16" t="n">
-        <v>126776.96</v>
-      </c>
-      <c r="G35" s="16" t="n">
-        <v>131848.04</v>
-      </c>
-      <c r="H35" s="16" t="n">
-        <v>137121.96</v>
-      </c>
-      <c r="I35" s="16" t="n">
-        <v>142606.83</v>
-      </c>
-      <c r="J35" s="16" t="n">
-        <v>660254.71</v>
+      <c r="B34" s="14" t="inlineStr"/>
+      <c r="C34" s="15" t="inlineStr"/>
+      <c r="D34" s="16" t="n">
+        <v>6147.27</v>
+      </c>
+      <c r="E34" s="16" t="n">
+        <v>73767.24000000001</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>76717.92999999999</v>
+      </c>
+      <c r="G34" s="16" t="n">
+        <v>79786.64999999999</v>
+      </c>
+      <c r="H34" s="16" t="n">
+        <v>82978.11</v>
+      </c>
+      <c r="I34" s="16" t="n">
+        <v>86297.24000000001</v>
+      </c>
+      <c r="J34" s="16" t="n">
+        <v>399547.17</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Pricing Assumptions</t>
+        </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Pricing Assumptions</t>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>us-east-1</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="B38" s="17" t="inlineStr">
-        <is>
-          <t>us-east-1</t>
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Inflation Rate/yr</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>4.0%</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>Inflation Rate/yr</t>
-        </is>
-      </c>
-      <c r="B39" s="18" t="inlineStr">
-        <is>
-          <t>4.0%</t>
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Hours/Month</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>730</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>Hours/Month</t>
-        </is>
-      </c>
-      <c r="B40" s="17" t="inlineStr">
-        <is>
-          <t>730</t>
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="B40" s="18" t="inlineStr">
+        <is>
+          <t>Multi-AZ (HA) for Prod/DR; Single-AZ for Pre-Prod + SIT + UAT</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>Deployment</t>
-        </is>
-      </c>
-      <c r="B41" s="18" t="inlineStr">
-        <is>
-          <t>Multi-AZ (HA) for Prod/DR; Single-AZ for Pre-Prod + SIT + UAT</t>
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Linux/RHEL</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>OS</t>
-        </is>
-      </c>
-      <c r="B42" s="17" t="inlineStr">
-        <is>
-          <t>Linux/RHEL</t>
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>EBS Type</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>gp3 (compute), io2 (SAN/DB)</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>EBS Type</t>
-        </is>
-      </c>
-      <c r="B43" s="18" t="inlineStr">
-        <is>
-          <t>gp3 (compute), io2 (SAN/DB)</t>
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Pricing Date</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>Pricing Date</t>
-        </is>
-      </c>
-      <c r="B44" s="17" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="10" t="inlineStr">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>DB Hosting</t>
         </is>
       </c>
-      <c r="B45" s="18" t="inlineStr">
+      <c r="B44" s="18" t="inlineStr">
         <is>
           <t>PostgreSQL=Self-Hosted EC2, SQL Server/Oracle=AWS RDS Managed</t>
         </is>
@@ -1855,14 +1817,14 @@
   <mergeCells count="10">
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A19:I19"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A37:I37"/>
     <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A27:I27"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A26:I26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1890,7 +1852,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Pre-Prod / SIT / UAT Environment  |  PNB  |  DB: PostgreSQL</t>
+          <t>Pre-Prod / SIT / UAT Environment  |  PAYTM  |  DB: PostgreSQL</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2547,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Disaster Recovery Environment  |  PNB  |  DB: PostgreSQL  |  Inflation: 4%/yr</t>
+          <t>Disaster Recovery Environment  |  PAYTM  |  DB: PostgreSQL  |  Inflation: 4%/yr</t>
         </is>
       </c>
     </row>
@@ -3422,14 +3384,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PUPM Summary – 5-Year Cost Analysis  |  PNB  |  24 Mar 2026  |  Inflation: 4.0%/yr</t>
+          <t>PUPM Summary – 5-Year Cost Analysis  |  PAYTM  |  09 Apr 2026  |  Inflation: 4.0%/yr</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PUPM Y1: $2.55  →  PUPM Y5: $2.40   |   Discount: 11%  |  Managed Services: 30%</t>
+          <t>PUPM Y1: $57.53  →  PUPM Y5: $53.78   |   Discount: 11%  |  Managed Services: 30%</t>
         </is>
       </c>
     </row>
@@ -3506,19 +3468,19 @@
       <c r="C5" s="10" t="inlineStr"/>
       <c r="D5" s="11" t="inlineStr"/>
       <c r="E5" s="12" t="n">
-        <v>10158.41</v>
+        <v>6147.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>10564.75</v>
+        <v>6393.16</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>10987.34</v>
+        <v>6648.89</v>
       </c>
       <c r="H5" s="12" t="n">
-        <v>11426.83</v>
+        <v>6914.84</v>
       </c>
       <c r="I5" s="12" t="n">
-        <v>11883.9</v>
+        <v>7191.44</v>
       </c>
     </row>
     <row r="6">
@@ -3834,19 +3796,19 @@
       <c r="C21" s="14" t="inlineStr"/>
       <c r="D21" s="15" t="inlineStr"/>
       <c r="E21" s="16" t="n">
-        <v>30706.1533</v>
+        <v>26695.0133</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>31894.0733</v>
+        <v>27722.4833</v>
       </c>
       <c r="G21" s="16" t="n">
-        <v>33129.4933</v>
+        <v>28791.0433</v>
       </c>
       <c r="H21" s="16" t="n">
-        <v>34414.3433</v>
+        <v>29902.3533</v>
       </c>
       <c r="I21" s="16" t="n">
-        <v>35750.5733</v>
+        <v>31058.1133</v>
       </c>
     </row>
     <row r="22">
@@ -3859,19 +3821,19 @@
       <c r="C22" s="7" t="inlineStr"/>
       <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="9" t="n">
-        <v>1201.4397</v>
+        <v>1044.4958</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>1247.9194</v>
+        <v>1084.6976</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>1296.2577</v>
+        <v>1126.5072</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>1346.53</v>
+        <v>1169.9894</v>
       </c>
       <c r="I22" s="9" t="n">
-        <v>1398.8127</v>
+        <v>1215.2108</v>
       </c>
     </row>
     <row r="23">
@@ -3886,19 +3848,19 @@
         <v>10000</v>
       </c>
       <c r="E23" s="22" t="n">
-        <v>382891.116</v>
+        <v>332874.1092</v>
       </c>
       <c r="F23" s="22" t="n">
-        <v>397703.9124</v>
+        <v>345686.1708</v>
       </c>
       <c r="G23" s="22" t="n">
-        <v>413109.012</v>
+        <v>359010.606</v>
       </c>
       <c r="H23" s="22" t="n">
-        <v>429130.4796</v>
+        <v>372868.1124</v>
       </c>
       <c r="I23" s="22" t="n">
-        <v>445792.632</v>
+        <v>387279.8892</v>
       </c>
     </row>
     <row r="24">
@@ -3911,19 +3873,19 @@
       <c r="C24" s="7" t="inlineStr"/>
       <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="9" t="n">
-        <v>19144.5558</v>
+        <v>16643.7055</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>19885.1956</v>
+        <v>17284.3085</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>20655.4506</v>
+        <v>17950.5303</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>21456.524</v>
+        <v>18643.4056</v>
       </c>
       <c r="I24" s="9" t="n">
-        <v>22289.6316</v>
+        <v>19363.9945</v>
       </c>
     </row>
     <row r="25">
@@ -3938,19 +3900,19 @@
         <v>10000</v>
       </c>
       <c r="E25" s="16" t="n">
-        <v>402035.6718</v>
+        <v>349517.8147</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>417589.108</v>
+        <v>362970.4793</v>
       </c>
       <c r="G25" s="16" t="n">
-        <v>433764.4626</v>
+        <v>376961.1363</v>
       </c>
       <c r="H25" s="16" t="n">
-        <v>450587.0036</v>
+        <v>391511.518</v>
       </c>
       <c r="I25" s="16" t="n">
-        <v>468082.2636</v>
+        <v>406643.8837</v>
       </c>
     </row>
     <row r="26">
@@ -3965,19 +3927,19 @@
         <v>1000</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>120610.7015</v>
+        <v>104855.3444</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>125276.7324</v>
+        <v>108891.1438</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>130129.3388</v>
+        <v>113088.3409</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>135176.1011</v>
+        <v>117453.4554</v>
       </c>
       <c r="I26" s="9" t="n">
-        <v>140424.6791</v>
+        <v>121993.1651</v>
       </c>
     </row>
     <row r="27">
@@ -3992,19 +3954,19 @@
         <v>11000</v>
       </c>
       <c r="E27" s="16" t="n">
-        <v>533646.3733</v>
+        <v>465373.1591</v>
       </c>
       <c r="F27" s="16" t="n">
-        <v>542865.8404</v>
+        <v>471861.6231</v>
       </c>
       <c r="G27" s="16" t="n">
-        <v>563893.8014</v>
+        <v>490049.4772</v>
       </c>
       <c r="H27" s="16" t="n">
-        <v>585763.1047</v>
+        <v>508964.9734</v>
       </c>
       <c r="I27" s="16" t="n">
-        <v>608506.9427</v>
+        <v>528637.0488</v>
       </c>
     </row>
     <row r="28">
@@ -4044,19 +4006,19 @@
         <v>11000</v>
       </c>
       <c r="E29" s="16" t="n">
-        <v>474945.2722</v>
+        <v>414182.1116</v>
       </c>
       <c r="F29" s="16" t="n">
-        <v>483150.598</v>
+        <v>419956.8446</v>
       </c>
       <c r="G29" s="16" t="n">
-        <v>501865.4832</v>
+        <v>436144.0347</v>
       </c>
       <c r="H29" s="16" t="n">
-        <v>521329.1632</v>
+        <v>452978.8263</v>
       </c>
       <c r="I29" s="16" t="n">
-        <v>541571.179</v>
+        <v>470486.9734</v>
       </c>
     </row>
     <row r="30" ht="6" customHeight="1">
@@ -4087,19 +4049,19 @@
       <c r="C32" s="10" t="inlineStr"/>
       <c r="D32" s="11" t="inlineStr"/>
       <c r="E32" s="12" t="n">
-        <v>15500</v>
+        <v>600</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>16275</v>
+        <v>630</v>
       </c>
       <c r="G32" s="12" t="n">
-        <v>17088</v>
+        <v>661</v>
       </c>
       <c r="H32" s="12" t="n">
-        <v>17943</v>
+        <v>694</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>18840</v>
+        <v>729</v>
       </c>
     </row>
     <row r="33" ht="26" customHeight="1">
@@ -4112,19 +4074,19 @@
       <c r="C33" s="24" t="inlineStr"/>
       <c r="D33" s="25" t="inlineStr"/>
       <c r="E33" s="26" t="n">
-        <v>2.5535</v>
+        <v>57.5253</v>
       </c>
       <c r="F33" s="26" t="n">
-        <v>2.4739</v>
+        <v>55.5498</v>
       </c>
       <c r="G33" s="26" t="n">
-        <v>2.4475</v>
+        <v>54.9854</v>
       </c>
       <c r="H33" s="26" t="n">
-        <v>2.4212</v>
+        <v>54.3923</v>
       </c>
       <c r="I33" s="26" t="n">
-        <v>2.3955</v>
+        <v>53.7822</v>
       </c>
     </row>
     <row r="34" ht="6" customHeight="1">
@@ -4191,22 +4153,22 @@
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>10158.41</v>
+        <v>6147.27</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>10564.75</v>
+        <v>6393.16</v>
       </c>
       <c r="E37" s="9" t="n">
-        <v>10987.34</v>
+        <v>6648.89</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>11426.83</v>
+        <v>6914.84</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>11883.9</v>
+        <v>7191.44</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>11004.246</v>
+        <v>6659.12</v>
       </c>
     </row>
     <row r="38">
@@ -4217,22 +4179,22 @@
         </is>
       </c>
       <c r="C38" s="12" t="n">
-        <v>30706.1533</v>
+        <v>26695.0133</v>
       </c>
       <c r="D38" s="12" t="n">
-        <v>31894.0733</v>
+        <v>27722.4833</v>
       </c>
       <c r="E38" s="12" t="n">
-        <v>33129.4933</v>
+        <v>28791.0433</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>34414.3433</v>
+        <v>29902.3533</v>
       </c>
       <c r="G38" s="12" t="n">
-        <v>35750.5733</v>
+        <v>31058.1133</v>
       </c>
       <c r="H38" s="12" t="n">
-        <v>33178.9273</v>
+        <v>28833.8013</v>
       </c>
     </row>
     <row r="39">
@@ -4243,22 +4205,22 @@
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>474945.2722</v>
+        <v>414182.1116</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>483150.598</v>
+        <v>419956.8446</v>
       </c>
       <c r="E39" s="9" t="n">
-        <v>501865.4832</v>
+        <v>436144.0347</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>521329.1632</v>
+        <v>452978.8263</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>541571.179</v>
+        <v>470486.9734</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>504572.33912</v>
+        <v>438749.75812</v>
       </c>
     </row>
     <row r="40">
@@ -4269,22 +4231,22 @@
         </is>
       </c>
       <c r="C40" s="12" t="n">
-        <v>15500</v>
+        <v>600</v>
       </c>
       <c r="D40" s="12" t="n">
-        <v>16275</v>
+        <v>630</v>
       </c>
       <c r="E40" s="12" t="n">
-        <v>17088</v>
+        <v>661</v>
       </c>
       <c r="F40" s="12" t="n">
-        <v>17943</v>
+        <v>694</v>
       </c>
       <c r="G40" s="12" t="n">
-        <v>18840</v>
+        <v>729</v>
       </c>
       <c r="H40" s="12" t="n">
-        <v>17129.2</v>
+        <v>662.8</v>
       </c>
     </row>
     <row r="41">
@@ -4295,22 +4257,22 @@
         </is>
       </c>
       <c r="C41" s="26" t="n">
-        <v>2.5535</v>
+        <v>57.5253</v>
       </c>
       <c r="D41" s="26" t="n">
-        <v>2.4739</v>
+        <v>55.5498</v>
       </c>
       <c r="E41" s="26" t="n">
-        <v>2.4475</v>
+        <v>54.9854</v>
       </c>
       <c r="F41" s="26" t="n">
-        <v>2.4212</v>
+        <v>54.3923</v>
       </c>
       <c r="G41" s="26" t="n">
-        <v>2.3955</v>
+        <v>53.7822</v>
       </c>
       <c r="H41" s="26" t="n">
-        <v>2.45832</v>
+        <v>55.247</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
@@ -4419,14 +4381,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>GCP Compute Engine Pricing — PNB</t>
+          <t>GCP Compute Engine Pricing — PAYTM</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>Region: us-central1  (US Central (Iowa))  ·  Generated: 24 Mar 2026  ·  All On-Demand prices  ·  GCP fallback rates</t>
+          <t>Region: us-central1  (US Central (Iowa))  ·  Generated: 09 Apr 2026  ·  All On-Demand prices  ·  GCP fallback rates</t>
         </is>
       </c>
     </row>
@@ -4482,10 +4444,10 @@
         <v>1.16832</v>
       </c>
       <c r="E5" s="34" t="n">
-        <v>5378.36</v>
+        <v>1792.79</v>
       </c>
       <c r="F5" s="34" t="n">
-        <v>64540.32</v>
+        <v>21513.48</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -4501,17 +4463,17 @@
       </c>
       <c r="C6" s="35" t="inlineStr">
         <is>
-          <t>n2-standard-8</t>
+          <t>n2-standard-16</t>
         </is>
       </c>
       <c r="D6" s="36" t="n">
-        <v>0.58416</v>
+        <v>1.16832</v>
       </c>
       <c r="E6" s="36" t="n">
-        <v>513.48</v>
+        <v>939.91</v>
       </c>
       <c r="F6" s="36" t="n">
-        <v>6161.76</v>
+        <v>11278.92</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -4527,17 +4489,17 @@
       </c>
       <c r="C7" s="33" t="inlineStr">
         <is>
-          <t>n2-standard-8</t>
+          <t>N/A (storage only)</t>
         </is>
       </c>
       <c r="D7" s="34" t="n">
-        <v>0.58416</v>
+        <v>0</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>1201.03</v>
+        <v>0</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>14412.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -4574,7 +4536,7 @@
       </c>
       <c r="B9" s="33" t="inlineStr">
         <is>
-          <t>Linux Nodes – Cluster (etcd+haproxy, pgbackrest)</t>
+          <t>Nodes – Cluster (etcd+haproxy, pgbackrest)</t>
         </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
@@ -4600,7 +4562,7 @@
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>Storage: SAN (Primary DB)</t>
+          <t>Storage: SAN (Primary PostgreSQL DB)</t>
         </is>
       </c>
       <c r="C10" s="35" t="inlineStr">
@@ -4612,10 +4574,10 @@
         <v>0</v>
       </c>
       <c r="E10" s="36" t="n">
-        <v>525</v>
+        <v>25</v>
       </c>
       <c r="F10" s="36" t="n">
-        <v>6300</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -4638,10 +4600,10 @@
         <v>0</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>737.5</v>
+        <v>25</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>8850</v>
+        <v>300</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -4898,10 +4860,10 @@
         <v>0</v>
       </c>
       <c r="E21" s="34" t="n">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="F21" s="34" t="n">
-        <v>960</v>
+        <v>708</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -4914,10 +4876,10 @@
       <c r="C22" s="38" t="n"/>
       <c r="D22" s="38" t="n"/>
       <c r="E22" s="39" t="n">
-        <v>15801.26</v>
+        <v>10207.59</v>
       </c>
       <c r="F22" s="39" t="n">
-        <v>189615.12</v>
+        <v>122491.08</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -4971,13 +4933,13 @@
         </is>
       </c>
       <c r="C26" s="36" t="n">
-        <v>15801.26</v>
+        <v>10207.59</v>
       </c>
       <c r="D26" s="36" t="n">
-        <v>189615.12</v>
+        <v>122491.08</v>
       </c>
       <c r="E26" s="36" t="n">
-        <v>189615.12</v>
+        <v>122491.08</v>
       </c>
       <c r="F26" s="42" t="inlineStr">
         <is>
@@ -4997,13 +4959,13 @@
         </is>
       </c>
       <c r="C27" s="34" t="n">
-        <v>16433.31</v>
+        <v>10615.89</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>197199.72</v>
+        <v>127390.68</v>
       </c>
       <c r="E27" s="34" t="n">
-        <v>386814.84</v>
+        <v>249881.76</v>
       </c>
       <c r="F27" s="43" t="inlineStr">
         <is>
@@ -5023,13 +4985,13 @@
         </is>
       </c>
       <c r="C28" s="36" t="n">
-        <v>17090.64</v>
+        <v>11040.53</v>
       </c>
       <c r="D28" s="36" t="n">
-        <v>205087.68</v>
+        <v>132486.36</v>
       </c>
       <c r="E28" s="36" t="n">
-        <v>591902.52</v>
+        <v>382368.12</v>
       </c>
       <c r="F28" s="42" t="inlineStr">
         <is>
@@ -5049,13 +5011,13 @@
         </is>
       </c>
       <c r="C29" s="34" t="n">
-        <v>17774.27</v>
+        <v>11482.15</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>213291.24</v>
+        <v>137785.8</v>
       </c>
       <c r="E29" s="34" t="n">
-        <v>805193.76</v>
+        <v>520153.92</v>
       </c>
       <c r="F29" s="43" t="inlineStr">
         <is>
@@ -5075,13 +5037,13 @@
         </is>
       </c>
       <c r="C30" s="36" t="n">
-        <v>18485.24</v>
+        <v>11941.44</v>
       </c>
       <c r="D30" s="36" t="n">
-        <v>221822.88</v>
+        <v>143297.28</v>
       </c>
       <c r="E30" s="36" t="n">
-        <v>1027016.64</v>
+        <v>663451.2</v>
       </c>
       <c r="F30" s="42" t="inlineStr">
         <is>
@@ -5105,7 +5067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5120,14 +5082,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="44" t="inlineStr">
         <is>
-          <t>AWS vs GCP Cost Comparison — PNB</t>
+          <t>AWS vs GCP Cost Comparison — PAYTM</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>AWS Region: us-east-1   |   GCP Region: us-central1   |   Generated: 24 Mar 2026   |   On-Demand pricing</t>
+          <t>AWS Region: us-east-1   |   GCP Region: us-central1   |   Generated: 09 Apr 2026   |   On-Demand pricing</t>
         </is>
       </c>
     </row>
@@ -5145,7 +5107,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>10158.41</v>
+        <v>6147.27</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5155,7 +5117,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>15801.26</v>
+        <v>10207.59</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -5165,7 +5127,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>5642.85</v>
+        <v>4060.32</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -5187,7 +5149,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>121900.92</v>
+        <v>73767.24000000001</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -5197,7 +5159,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>189615.12</v>
+        <v>122491.08</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -5207,7 +5169,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>660254.76</v>
+        <v>399547.2</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -5217,7 +5179,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>1027016.64</v>
+        <v>663451.2</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -5227,7 +5189,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>366761.88</v>
+        <v>263904</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -5320,17 +5282,17 @@
         </is>
       </c>
       <c r="B19" s="36" t="n">
-        <v>337.35</v>
+        <v>328.35</v>
       </c>
       <c r="C19" s="36" t="n">
         <v>429.61</v>
       </c>
       <c r="D19" s="36" t="n">
-        <v>92.26000000000001</v>
+        <v>101.26</v>
       </c>
       <c r="E19" s="42" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="F19" s="49" t="inlineStr">
@@ -5351,17 +5313,17 @@
         </is>
       </c>
       <c r="B20" s="34" t="n">
-        <v>4605.48</v>
+        <v>1836.84</v>
       </c>
       <c r="C20" s="34" t="n">
-        <v>7165.87</v>
+        <v>2805.7</v>
       </c>
       <c r="D20" s="34" t="n">
-        <v>2560.39</v>
+        <v>968.86</v>
       </c>
       <c r="E20" s="43" t="inlineStr">
         <is>
-          <t>35.7%</t>
+          <t>34.5%</t>
         </is>
       </c>
       <c r="F20" s="49" t="inlineStr">
@@ -5382,10 +5344,10 @@
         </is>
       </c>
       <c r="B21" s="36" t="n">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="C21" s="36" t="n">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="D21" s="36" t="n">
         <v>0</v>
@@ -5413,17 +5375,17 @@
         </is>
       </c>
       <c r="B22" s="34" t="n">
-        <v>3916.28</v>
+        <v>3416.28</v>
       </c>
       <c r="C22" s="34" t="n">
-        <v>7030.58</v>
+        <v>6530.58</v>
       </c>
       <c r="D22" s="34" t="n">
         <v>3114.3</v>
       </c>
       <c r="E22" s="43" t="inlineStr">
         <is>
-          <t>44.3%</t>
+          <t>47.7%</t>
         </is>
       </c>
       <c r="F22" s="49" t="inlineStr">
@@ -5444,10 +5406,10 @@
         </is>
       </c>
       <c r="B23" s="36" t="n">
-        <v>737.5</v>
+        <v>25</v>
       </c>
       <c r="C23" s="36" t="n">
-        <v>737.5</v>
+        <v>25</v>
       </c>
       <c r="D23" s="36" t="n">
         <v>0</v>
@@ -5546,126 +5508,26 @@
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="43" t="inlineStr">
         <is>
-          <t>Year 1</t>
+          <t>Year 5</t>
         </is>
       </c>
       <c r="B28" s="52" t="n">
-        <v>10158.41</v>
+        <v>7191.44</v>
       </c>
       <c r="C28" s="34" t="n">
-        <v>15801.26</v>
+        <v>11941.44</v>
       </c>
       <c r="D28" s="34" t="n">
-        <v>121900.92</v>
+        <v>86297.28</v>
       </c>
       <c r="E28" s="34" t="n">
-        <v>189615.12</v>
+        <v>143297.28</v>
       </c>
       <c r="F28" s="34" t="n">
-        <v>121900.92</v>
+        <v>399547.2</v>
       </c>
       <c r="G28" s="34" t="n">
-        <v>189615.12</v>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="42" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B29" s="52" t="n">
-        <v>10564.75</v>
-      </c>
-      <c r="C29" s="36" t="n">
-        <v>16433.31</v>
-      </c>
-      <c r="D29" s="36" t="n">
-        <v>126777</v>
-      </c>
-      <c r="E29" s="36" t="n">
-        <v>197199.72</v>
-      </c>
-      <c r="F29" s="36" t="n">
-        <v>248677.92</v>
-      </c>
-      <c r="G29" s="36" t="n">
-        <v>386814.84</v>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="43" t="inlineStr">
-        <is>
-          <t>Year 3</t>
-        </is>
-      </c>
-      <c r="B30" s="52" t="n">
-        <v>10987.34</v>
-      </c>
-      <c r="C30" s="34" t="n">
-        <v>17090.64</v>
-      </c>
-      <c r="D30" s="34" t="n">
-        <v>131848.08</v>
-      </c>
-      <c r="E30" s="34" t="n">
-        <v>205087.68</v>
-      </c>
-      <c r="F30" s="34" t="n">
-        <v>380526</v>
-      </c>
-      <c r="G30" s="34" t="n">
-        <v>591902.52</v>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="42" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B31" s="52" t="n">
-        <v>11426.83</v>
-      </c>
-      <c r="C31" s="36" t="n">
-        <v>17774.27</v>
-      </c>
-      <c r="D31" s="36" t="n">
-        <v>137121.96</v>
-      </c>
-      <c r="E31" s="36" t="n">
-        <v>213291.24</v>
-      </c>
-      <c r="F31" s="36" t="n">
-        <v>517647.96</v>
-      </c>
-      <c r="G31" s="36" t="n">
-        <v>805193.76</v>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="43" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B32" s="52" t="n">
-        <v>11883.9</v>
-      </c>
-      <c r="C32" s="34" t="n">
-        <v>18485.24</v>
-      </c>
-      <c r="D32" s="34" t="n">
-        <v>142606.8</v>
-      </c>
-      <c r="E32" s="34" t="n">
-        <v>221822.88</v>
-      </c>
-      <c r="F32" s="34" t="n">
-        <v>660254.76</v>
-      </c>
-      <c r="G32" s="34" t="n">
-        <v>1027016.64</v>
+        <v>663451.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated all the changes about location drop down, formatted chatbot, added more instance families.
</commit_message>
<xml_diff>
--- a/reports/aws_pricing_forecast.xlsx
+++ b/reports/aws_pricing_forecast.xlsx
@@ -740,14 +740,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AWS 5-Year Cost Forecast  |  Apple FCU  |  16 Apr 2026  |  Inflation: 4.0%/yr</t>
+          <t>AWS 5-Year Cost Forecast  |  RHB  |  20 Apr 2026  |  Inflation: 4.0%/yr</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Base Monthly: $10,999.37  |  Annual Y1: $131,992.44  |  3-Year: $395,977.32</t>
+          <t>Base Monthly: $10,296.72  |  Annual Y1: $123,560.64  |  3-Year: $370,681.92</t>
         </is>
       </c>
     </row>
@@ -936,29 +936,29 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>m5.large</t>
+          <t>c6i.large</t>
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>94.08</v>
+        <v>87.20999999999999</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>1128.96</v>
+        <v>1046.52</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1174.12</v>
+        <v>1088.38</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>1221.08</v>
+        <v>1131.92</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>1269.93</v>
+        <v>1177.19</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>1320.72</v>
+        <v>1224.28</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>6114.81</v>
+        <v>5668.29</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -1016,25 +1016,25 @@
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>51.2</v>
+        <v>56.32</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>614.4</v>
+        <v>675.84</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>638.98</v>
+        <v>702.87</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>664.54</v>
+        <v>730.99</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>691.12</v>
+        <v>760.23</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>718.76</v>
+        <v>790.64</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>3327.8</v>
+        <v>3660.57</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -1095,29 +1095,29 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>m5.4xlarge</t>
+          <t>c6i.4xlarge</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>3486.72</v>
+        <v>3054</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>41840.64</v>
+        <v>36648</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>43514.27</v>
+        <v>38113.92</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>45254.84</v>
+        <v>39638.48</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>47065.03</v>
+        <v>41224.02</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>48947.63</v>
+        <v>42872.98</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>226622.41</v>
+        <v>198497.4</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -1133,29 +1133,29 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>m5.4xlarge</t>
+          <t>c6i.2xlarge</t>
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>601.6</v>
+        <v>576.58</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>7219.2</v>
+        <v>6918.96</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>7507.97</v>
+        <v>7195.72</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>7808.29</v>
+        <v>7483.55</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>8120.62</v>
+        <v>7782.89</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>8445.440000000001</v>
+        <v>8094.2</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>39101.52</v>
+        <v>37475.32</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -1171,29 +1171,29 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>m5.4xlarge</t>
+          <t>c6i.4xlarge</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>1285.12</v>
+        <v>576.58</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>15421.44</v>
+        <v>6918.96</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>16038.3</v>
+        <v>7195.72</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>16679.83</v>
+        <v>7483.55</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>17347.02</v>
+        <v>7782.89</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>18040.9</v>
+        <v>8094.2</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>83527.49000000001</v>
+        <v>37475.32</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -1303,25 +1303,25 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>2991.36</v>
+        <v>3290.5</v>
       </c>
       <c r="E21" s="12" t="n">
-        <v>35896.32</v>
+        <v>39486</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>37332.17</v>
+        <v>41065.44</v>
       </c>
       <c r="G21" s="12" t="n">
-        <v>38825.46</v>
+        <v>42708.06</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>40378.48</v>
+        <v>44416.38</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>41993.62</v>
+        <v>46193.04</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>194426.05</v>
+        <v>213868.92</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -1341,25 +1341,25 @@
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>399.92</v>
+        <v>439.91</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>4799.04</v>
+        <v>5278.92</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>4991</v>
+        <v>5490.08</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>5190.64</v>
+        <v>5709.68</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>5398.27</v>
+        <v>5938.07</v>
       </c>
       <c r="I22" s="9" t="n">
-        <v>5614.2</v>
+        <v>6175.59</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>25993.15</v>
+        <v>28592.34</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -1379,25 +1379,25 @@
         </is>
       </c>
       <c r="D23" s="12" t="n">
-        <v>525</v>
+        <v>577.5</v>
       </c>
       <c r="E23" s="12" t="n">
-        <v>6300</v>
+        <v>6930</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>6552</v>
+        <v>7207.2</v>
       </c>
       <c r="G23" s="12" t="n">
-        <v>6814.08</v>
+        <v>7495.49</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>7086.64</v>
+        <v>7795.31</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>7370.11</v>
+        <v>8107.12</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>34122.83</v>
+        <v>37535.12</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -1424,25 +1424,25 @@
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>737.5</v>
+        <v>811.25</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>8850</v>
+        <v>9735</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>9204</v>
+        <v>10124.4</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>9572.16</v>
+        <v>10529.38</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>9955.049999999999</v>
+        <v>10950.55</v>
       </c>
       <c r="I25" s="9" t="n">
-        <v>10353.25</v>
+        <v>11388.57</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>47934.46</v>
+        <v>52727.9</v>
       </c>
     </row>
     <row r="27">
@@ -1507,25 +1507,25 @@
         </is>
       </c>
       <c r="D29" s="12" t="n">
-        <v>337.35</v>
+        <v>335.6</v>
       </c>
       <c r="E29" s="12" t="n">
-        <v>4048.2</v>
+        <v>4027.2</v>
       </c>
       <c r="F29" s="12" t="n">
-        <v>4210.13</v>
+        <v>4188.29</v>
       </c>
       <c r="G29" s="12" t="n">
-        <v>4378.53</v>
+        <v>4355.82</v>
       </c>
       <c r="H29" s="12" t="n">
-        <v>4553.67</v>
+        <v>4530.05</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>4735.82</v>
+        <v>4711.25</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>21926.35</v>
+        <v>21812.61</v>
       </c>
     </row>
     <row r="30">
@@ -1545,25 +1545,25 @@
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>5446.44</v>
+        <v>4280.16</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>65357.28</v>
+        <v>51361.92</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>67971.57000000001</v>
+        <v>53416.4</v>
       </c>
       <c r="G30" s="9" t="n">
-        <v>70690.42999999999</v>
+        <v>55553.05</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>73518.05</v>
+        <v>57775.17</v>
       </c>
       <c r="I30" s="9" t="n">
-        <v>76458.77</v>
+        <v>60086.18</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>353996.1</v>
+        <v>278192.72</v>
       </c>
     </row>
     <row r="31">
@@ -1621,25 +1621,25 @@
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>3916.28</v>
+        <v>4307.91</v>
       </c>
       <c r="E32" s="9" t="n">
-        <v>46995.36</v>
+        <v>51694.92</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>48875.17</v>
+        <v>53762.72</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>50830.18</v>
+        <v>55913.23</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>52863.39</v>
+        <v>58149.75</v>
       </c>
       <c r="I32" s="9" t="n">
-        <v>54977.92</v>
+        <v>60475.74</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>254542.02</v>
+        <v>279996.36</v>
       </c>
     </row>
     <row r="33">
@@ -1659,25 +1659,25 @@
         </is>
       </c>
       <c r="D33" s="12" t="n">
-        <v>737.5</v>
+        <v>811.25</v>
       </c>
       <c r="E33" s="12" t="n">
-        <v>8850</v>
+        <v>9735</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>9204</v>
+        <v>10124.4</v>
       </c>
       <c r="G33" s="12" t="n">
-        <v>9572.16</v>
+        <v>10529.38</v>
       </c>
       <c r="H33" s="12" t="n">
-        <v>9955.049999999999</v>
+        <v>10950.55</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>10353.25</v>
+        <v>11388.57</v>
       </c>
       <c r="J33" s="12" t="n">
-        <v>47934.46</v>
+        <v>52727.9</v>
       </c>
     </row>
     <row r="34">
@@ -1727,25 +1727,25 @@
       <c r="B35" s="14" t="inlineStr"/>
       <c r="C35" s="15" t="inlineStr"/>
       <c r="D35" s="16" t="n">
-        <v>10999.37</v>
+        <v>10296.72</v>
       </c>
       <c r="E35" s="16" t="n">
-        <v>131992.44</v>
+        <v>123560.64</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>137272.14</v>
+        <v>128503.07</v>
       </c>
       <c r="G35" s="16" t="n">
-        <v>142763.02</v>
+        <v>133643.19</v>
       </c>
       <c r="H35" s="16" t="n">
-        <v>148473.54</v>
+        <v>138988.92</v>
       </c>
       <c r="I35" s="16" t="n">
-        <v>154412.49</v>
+        <v>144548.47</v>
       </c>
       <c r="J35" s="16" t="n">
-        <v>714913.63</v>
+        <v>669244.29</v>
       </c>
     </row>
     <row r="37">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>us-east-1</t>
+          <t>ap-southeast-5</t>
         </is>
       </c>
     </row>
@@ -1890,14 +1890,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Pre-Prod / SIT / UAT Environment  |  Apple FCU  |  DB: PostgreSQL</t>
+          <t>Pre-Prod / SIT / UAT Environment  |  RHB  |  DB: PostgreSQL</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Monthly: $13,262.04   |   Annual: $159,144.48</t>
+          <t>Monthly: $13,426.83   |   Annual: $161,121.96</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>m5.4xlarge</t>
+          <t>c6i.4xlarge</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
@@ -2014,11 +2014,11 @@
         <v>19</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>2338.56</v>
+        <v>2051.49</v>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>4× m5.4xlarge @ $0.7680/hr + 300GB EBS</t>
+          <t>4× c6i.4xlarge @ $0.6664/hr + 300GB EBS</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>m5.2xlarge</t>
+          <t>c6i.2xlarge</t>
         </is>
       </c>
       <c r="E7" s="8" t="n">
@@ -2048,11 +2048,11 @@
         <v>16</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>321.28</v>
+        <v>288.29</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>1× m5.2xlarge @ $0.3840/hr + 512GB EBS</t>
+          <t>1× c6i.2xlarge @ $0.3332/hr + 512GB EBS</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>m5.8xlarge</t>
+          <t>c6i.12xlarge</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
@@ -2089,11 +2089,11 @@
         <v>96</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>1145.28</v>
+        <v>1485.82</v>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>1× m5.8xlarge @ $1.5360/hr + 300GB EBS</t>
+          <t>1× c6i.12xlarge @ $1.9992/hr + 300GB EBS</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>105</v>
+        <v>115.5</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
@@ -2213,7 +2213,7 @@
         <v>16</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>121.18</v>
+        <v>133.3</v>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
@@ -2330,7 +2330,7 @@
         <v>4</v>
       </c>
       <c r="G18" s="12" t="n">
-        <v>54.37</v>
+        <v>61.08</v>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="G19" s="9" t="n">
-        <v>51.2</v>
+        <v>56.32</v>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
@@ -2478,7 +2478,7 @@
       <c r="E24" s="15" t="inlineStr"/>
       <c r="F24" s="15" t="inlineStr"/>
       <c r="G24" s="16" t="n">
-        <v>13262.04</v>
+        <v>13426.83</v>
       </c>
       <c r="H24" s="15" t="inlineStr"/>
     </row>
@@ -2521,14 +2521,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Disaster Recovery Environment  |  Apple FCU  |  DB: PostgreSQL  |  Inflation: 4%/yr</t>
+          <t>Disaster Recovery Environment  |  RHB  |  DB: PostgreSQL  |  Inflation: 4%/yr</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Monthly: $8,585.73   |   Annual: $103,028.76   |   5-Year Total: $580,358.48</t>
+          <t>Monthly: $10,531.08   |   Annual: $126,372.96   |   5-Year Total: $711,855.78</t>
         </is>
       </c>
     </row>
@@ -2589,22 +2589,22 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>107149.91</v>
+        <v>131427.88</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>111435.91</v>
+        <v>136684.99</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>115893.34</v>
+        <v>142152.39</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>120529.08</v>
+        <v>147838.49</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>125350.24</v>
+        <v>153752.03</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>580358.48</v>
+        <v>711855.78</v>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
@@ -2739,11 +2739,11 @@
         <v>19</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>3486.72</v>
+        <v>4343.65</v>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>6× m5.4xlarge @ $0.7680/hr + 256GB EBS</t>
+          <t>6× m5.4xlarge @ $0.9600/hr + 256GB EBS</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr"/>
@@ -2774,11 +2774,11 @@
         <v>16</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>642.5599999999999</v>
+        <v>793.37</v>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>2× m5.2xlarge @ $0.3840/hr + 512GB EBS</t>
+          <t>2× m5.2xlarge @ $0.4800/hr + 512GB EBS</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr"/>
@@ -2816,11 +2816,11 @@
         <v>136</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>3411.84</v>
+        <v>4259.04</v>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>2× m5.12xlarge @ $2.3040/hr + 300GB EBS</t>
+          <t>2× m5.12xlarge @ $2.8800/hr + 300GB EBS</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr"/>
@@ -2855,7 +2855,7 @@
         </is>
       </c>
       <c r="G15" s="9" t="n">
-        <v>315</v>
+        <v>355.95</v>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
@@ -2943,7 +2943,7 @@
         <v>16</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>242.36</v>
+        <v>273.87</v>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
@@ -3063,7 +3063,7 @@
         <v>4</v>
       </c>
       <c r="G23" s="12" t="n">
-        <v>54.37</v>
+        <v>65.66</v>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
@@ -3102,7 +3102,7 @@
         </is>
       </c>
       <c r="G24" s="9" t="n">
-        <v>51.2</v>
+        <v>57.86</v>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
@@ -3215,7 +3215,7 @@
       <c r="E29" s="15" t="inlineStr"/>
       <c r="F29" s="15" t="inlineStr"/>
       <c r="G29" s="16" t="n">
-        <v>8585.73</v>
+        <v>10531.08</v>
       </c>
       <c r="H29" s="15" t="inlineStr"/>
       <c r="I29" s="15" t="inlineStr"/>
@@ -3261,14 +3261,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PUPM Summary – 5-Year Cost Analysis  |  Apple FCU  |  16 Apr 2026  |  Inflation: 4.0%/yr</t>
+          <t>PUPM Summary – 5-Year Cost Analysis  |  RHB  |  20 Apr 2026  |  Inflation: 4.0%/yr</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PUPM Y1: $2.81  →  PUPM Y5: $2.64   |   Discount: 11%  |  Managed Services: 30%</t>
+          <t>PUPM Y1: $2.92  →  PUPM Y5: $2.75   |   Discount: 11%  |  Managed Services: 30%</t>
         </is>
       </c>
     </row>
@@ -3345,19 +3345,19 @@
       <c r="C5" s="10" t="inlineStr"/>
       <c r="D5" s="11" t="inlineStr"/>
       <c r="E5" s="12" t="n">
-        <v>10999.37</v>
+        <v>10296.72</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>11439.34</v>
+        <v>10708.59</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>11896.92</v>
+        <v>11136.93</v>
       </c>
       <c r="H5" s="12" t="n">
-        <v>12372.8</v>
+        <v>11582.41</v>
       </c>
       <c r="I5" s="12" t="n">
-        <v>12867.71</v>
+        <v>12045.71</v>
       </c>
     </row>
     <row r="6">
@@ -3370,19 +3370,19 @@
       <c r="C6" s="7" t="inlineStr"/>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="9" t="n">
-        <v>8585.73</v>
+        <v>10531.08</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>8929.16</v>
+        <v>10952.32</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9286.33</v>
+        <v>11390.42</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>9657.780000000001</v>
+        <v>11846.03</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>10044.09</v>
+        <v>12319.87</v>
       </c>
     </row>
     <row r="7">
@@ -3395,19 +3395,19 @@
       <c r="C7" s="10" t="inlineStr"/>
       <c r="D7" s="11" t="inlineStr"/>
       <c r="E7" s="12" t="n">
-        <v>13262.04</v>
+        <v>13426.83</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>13792.52</v>
+        <v>13963.9</v>
       </c>
       <c r="G7" s="12" t="n">
-        <v>14344.22</v>
+        <v>14522.46</v>
       </c>
       <c r="H7" s="12" t="n">
-        <v>14917.99</v>
+        <v>15103.36</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>15514.71</v>
+        <v>15707.49</v>
       </c>
     </row>
     <row r="8">
@@ -3673,19 +3673,19 @@
       <c r="C21" s="14" t="inlineStr"/>
       <c r="D21" s="15" t="inlineStr"/>
       <c r="E21" s="16" t="n">
-        <v>33855.47330000001</v>
+        <v>35262.9633</v>
       </c>
       <c r="F21" s="16" t="n">
-        <v>35169.35330000001</v>
+        <v>36633.1433</v>
       </c>
       <c r="G21" s="16" t="n">
-        <v>36535.80330000001</v>
+        <v>38058.1433</v>
       </c>
       <c r="H21" s="16" t="n">
-        <v>37956.90330000001</v>
+        <v>39540.13330000001</v>
       </c>
       <c r="I21" s="16" t="n">
-        <v>39434.8433</v>
+        <v>41081.40330000001</v>
       </c>
     </row>
     <row r="22">
@@ -3698,19 +3698,19 @@
       <c r="C22" s="7" t="inlineStr"/>
       <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="9" t="n">
-        <v>1324.6631</v>
+        <v>1379.734</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>1376.0713</v>
+        <v>1433.345</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>1429.5364</v>
+        <v>1489.101</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>1485.1398</v>
+        <v>1547.0868</v>
       </c>
       <c r="I22" s="9" t="n">
-        <v>1542.9671</v>
+        <v>1607.3921</v>
       </c>
     </row>
     <row r="23">
@@ -3725,19 +3725,19 @@
         <v>10000</v>
       </c>
       <c r="E23" s="22" t="n">
-        <v>422161.6368</v>
+        <v>439712.3676</v>
       </c>
       <c r="F23" s="22" t="n">
-        <v>438545.0952</v>
+        <v>456797.8596</v>
       </c>
       <c r="G23" s="22" t="n">
-        <v>455584.0764</v>
+        <v>474566.9316</v>
       </c>
       <c r="H23" s="22" t="n">
-        <v>473304.5172</v>
+        <v>493046.6412</v>
       </c>
       <c r="I23" s="22" t="n">
-        <v>491733.7248</v>
+        <v>512265.5448</v>
       </c>
     </row>
     <row r="24">
@@ -3750,19 +3750,19 @@
       <c r="C24" s="7" t="inlineStr"/>
       <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="9" t="n">
-        <v>21108.0818</v>
+        <v>21985.6184</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>21927.2548</v>
+        <v>22839.893</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>22779.2038</v>
+        <v>23728.3466</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>23665.2259</v>
+        <v>24652.3321</v>
       </c>
       <c r="I24" s="9" t="n">
-        <v>24586.6862</v>
+        <v>25613.2772</v>
       </c>
     </row>
     <row r="25">
@@ -3777,19 +3777,19 @@
         <v>10000</v>
       </c>
       <c r="E25" s="16" t="n">
-        <v>443269.7186</v>
+        <v>461697.986</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>460472.35</v>
+        <v>479637.7526</v>
       </c>
       <c r="G25" s="16" t="n">
-        <v>478363.2802</v>
+        <v>498295.2782</v>
       </c>
       <c r="H25" s="16" t="n">
-        <v>496969.7431</v>
+        <v>517698.9733</v>
       </c>
       <c r="I25" s="16" t="n">
-        <v>516320.411</v>
+        <v>537878.822</v>
       </c>
     </row>
     <row r="26">
@@ -3804,19 +3804,19 @@
         <v>1000</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>132980.9156</v>
+        <v>138509.3958</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>138141.705</v>
+        <v>143891.3258</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>143508.9841</v>
+        <v>149488.5835</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>149090.9229</v>
+        <v>155309.692</v>
       </c>
       <c r="I26" s="9" t="n">
-        <v>154896.1233</v>
+        <v>161363.6466</v>
       </c>
     </row>
     <row r="27">
@@ -3831,19 +3831,19 @@
         <v>11000</v>
       </c>
       <c r="E27" s="16" t="n">
-        <v>587250.6342</v>
+        <v>611207.3818</v>
       </c>
       <c r="F27" s="16" t="n">
-        <v>598614.0550000001</v>
+        <v>623529.0784</v>
       </c>
       <c r="G27" s="16" t="n">
-        <v>621872.2643</v>
+        <v>647783.8617</v>
       </c>
       <c r="H27" s="16" t="n">
-        <v>646060.666</v>
+        <v>673008.6653</v>
       </c>
       <c r="I27" s="16" t="n">
-        <v>671216.5343000001</v>
+        <v>699242.4686</v>
       </c>
     </row>
     <row r="28">
@@ -3883,19 +3883,19 @@
         <v>11000</v>
       </c>
       <c r="E29" s="16" t="n">
-        <v>522653.0644</v>
+        <v>543974.5698000001</v>
       </c>
       <c r="F29" s="16" t="n">
-        <v>532766.509</v>
+        <v>554940.8798</v>
       </c>
       <c r="G29" s="16" t="n">
-        <v>553466.3152</v>
+        <v>576527.6369</v>
       </c>
       <c r="H29" s="16" t="n">
-        <v>574993.9926999999</v>
+        <v>598977.7121</v>
       </c>
       <c r="I29" s="16" t="n">
-        <v>597382.7155</v>
+        <v>622325.7971</v>
       </c>
     </row>
     <row r="30" ht="6" customHeight="1">
@@ -3951,19 +3951,19 @@
       <c r="C33" s="24" t="inlineStr"/>
       <c r="D33" s="25" t="inlineStr"/>
       <c r="E33" s="26" t="n">
-        <v>2.81</v>
+        <v>2.9246</v>
       </c>
       <c r="F33" s="26" t="n">
-        <v>2.7279</v>
+        <v>2.8415</v>
       </c>
       <c r="G33" s="26" t="n">
-        <v>2.6991</v>
+        <v>2.8116</v>
       </c>
       <c r="H33" s="26" t="n">
-        <v>2.6705</v>
+        <v>2.7819</v>
       </c>
       <c r="I33" s="26" t="n">
-        <v>2.6424</v>
+        <v>2.7527</v>
       </c>
     </row>
     <row r="34" ht="6" customHeight="1">
@@ -4030,22 +4030,22 @@
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>10999.37</v>
+        <v>10296.72</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>11439.34</v>
+        <v>10708.59</v>
       </c>
       <c r="E37" s="9" t="n">
-        <v>11896.92</v>
+        <v>11136.93</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>12372.8</v>
+        <v>11582.41</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>12867.71</v>
+        <v>12045.71</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>11915.228</v>
+        <v>11154.072</v>
       </c>
     </row>
     <row r="38">
@@ -4056,22 +4056,22 @@
         </is>
       </c>
       <c r="C38" s="12" t="n">
-        <v>33855.47330000001</v>
+        <v>35262.9633</v>
       </c>
       <c r="D38" s="12" t="n">
-        <v>35169.35330000001</v>
+        <v>36633.1433</v>
       </c>
       <c r="E38" s="12" t="n">
-        <v>36535.80330000001</v>
+        <v>38058.1433</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>37956.90330000001</v>
+        <v>39540.13330000001</v>
       </c>
       <c r="G38" s="12" t="n">
-        <v>39434.8433</v>
+        <v>41081.40330000001</v>
       </c>
       <c r="H38" s="12" t="n">
-        <v>36590.47530000001</v>
+        <v>38115.15730000001</v>
       </c>
     </row>
     <row r="39">
@@ -4082,22 +4082,22 @@
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>522653.0644</v>
+        <v>543974.5698000001</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>532766.509</v>
+        <v>554940.8798</v>
       </c>
       <c r="E39" s="9" t="n">
-        <v>553466.3152</v>
+        <v>576527.6369</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>574993.9926999999</v>
+        <v>598977.7121</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>597382.7155</v>
+        <v>622325.7971</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>556252.51936</v>
+        <v>579349.31914</v>
       </c>
     </row>
     <row r="40">
@@ -4134,22 +4134,22 @@
         </is>
       </c>
       <c r="C41" s="26" t="n">
-        <v>2.81</v>
+        <v>2.9246</v>
       </c>
       <c r="D41" s="26" t="n">
-        <v>2.7279</v>
+        <v>2.8415</v>
       </c>
       <c r="E41" s="26" t="n">
-        <v>2.6991</v>
+        <v>2.8116</v>
       </c>
       <c r="F41" s="26" t="n">
-        <v>2.6705</v>
+        <v>2.7819</v>
       </c>
       <c r="G41" s="26" t="n">
-        <v>2.6424</v>
+        <v>2.7527</v>
       </c>
       <c r="H41" s="26" t="n">
-        <v>2.70998</v>
+        <v>2.82246</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
@@ -4258,14 +4258,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>GCP Compute Engine Pricing — Apple FCU</t>
+          <t>GCP Compute Engine Pricing — RHB</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>Region: us-central1  (US Central (Iowa))  ·  Generated: 16 Apr 2026  ·  All On-Demand prices  ·  GCP fallback rates</t>
+          <t>Region: us-central1  (US Central (Iowa))  ·  Generated: 20 Apr 2026  ·  All On-Demand prices  ·  GCP fallback rates</t>
         </is>
       </c>
     </row>
@@ -4340,17 +4340,17 @@
       </c>
       <c r="C6" s="35" t="inlineStr">
         <is>
-          <t>n2-standard-16</t>
+          <t>n2-standard-8</t>
         </is>
       </c>
       <c r="D6" s="36" t="n">
-        <v>1.16832</v>
+        <v>0.58416</v>
       </c>
       <c r="E6" s="36" t="n">
-        <v>939.91</v>
+        <v>1026.95</v>
       </c>
       <c r="F6" s="36" t="n">
-        <v>11278.92</v>
+        <v>12323.4</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -4373,10 +4373,10 @@
         <v>1.16832</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>2053.91</v>
+        <v>1026.95</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>24646.92</v>
+        <v>12323.4</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -4753,10 +4753,10 @@
       <c r="C22" s="38" t="n"/>
       <c r="D22" s="38" t="n"/>
       <c r="E22" s="39" t="n">
-        <v>17080.57</v>
+        <v>16140.65</v>
       </c>
       <c r="F22" s="39" t="n">
-        <v>204966.84</v>
+        <v>193687.8</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -4810,13 +4810,13 @@
         </is>
       </c>
       <c r="C26" s="36" t="n">
-        <v>17080.57</v>
+        <v>16140.65</v>
       </c>
       <c r="D26" s="36" t="n">
-        <v>204966.84</v>
+        <v>193687.8</v>
       </c>
       <c r="E26" s="36" t="n">
-        <v>204966.84</v>
+        <v>193687.8</v>
       </c>
       <c r="F26" s="42" t="inlineStr">
         <is>
@@ -4836,13 +4836,13 @@
         </is>
       </c>
       <c r="C27" s="34" t="n">
-        <v>17763.79</v>
+        <v>16786.28</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>213165.48</v>
+        <v>201435.36</v>
       </c>
       <c r="E27" s="34" t="n">
-        <v>418132.32</v>
+        <v>395123.16</v>
       </c>
       <c r="F27" s="43" t="inlineStr">
         <is>
@@ -4862,13 +4862,13 @@
         </is>
       </c>
       <c r="C28" s="36" t="n">
-        <v>18474.34</v>
+        <v>17457.73</v>
       </c>
       <c r="D28" s="36" t="n">
-        <v>221692.08</v>
+        <v>209492.76</v>
       </c>
       <c r="E28" s="36" t="n">
-        <v>639824.4</v>
+        <v>604615.92</v>
       </c>
       <c r="F28" s="42" t="inlineStr">
         <is>
@@ -4888,13 +4888,13 @@
         </is>
       </c>
       <c r="C29" s="34" t="n">
-        <v>19213.32</v>
+        <v>18156.04</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>230559.84</v>
+        <v>217872.48</v>
       </c>
       <c r="E29" s="34" t="n">
-        <v>870384.24</v>
+        <v>822488.4</v>
       </c>
       <c r="F29" s="43" t="inlineStr">
         <is>
@@ -4914,13 +4914,13 @@
         </is>
       </c>
       <c r="C30" s="36" t="n">
-        <v>19981.85</v>
+        <v>18882.28</v>
       </c>
       <c r="D30" s="36" t="n">
-        <v>239782.2</v>
+        <v>226587.36</v>
       </c>
       <c r="E30" s="36" t="n">
-        <v>1110166.44</v>
+        <v>1049075.76</v>
       </c>
       <c r="F30" s="42" t="inlineStr">
         <is>
@@ -4959,14 +4959,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="44" t="inlineStr">
         <is>
-          <t>AWS vs GCP Cost Comparison — Apple FCU</t>
+          <t>AWS vs GCP Cost Comparison — RHB</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>AWS Region: us-east-1   |   GCP Region: us-central1   |   Generated: 16 Apr 2026   |   On-Demand pricing</t>
+          <t>AWS Region: ap-southeast-5   |   GCP Region: us-central1   |   Generated: 20 Apr 2026   |   On-Demand pricing</t>
         </is>
       </c>
     </row>
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>10999.37</v>
+        <v>10296.72</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -4994,7 +4994,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>17080.57</v>
+        <v>16140.65</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -5004,7 +5004,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>6081.2</v>
+        <v>5843.93</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -5026,7 +5026,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>131992.44</v>
+        <v>123560.64</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -5036,7 +5036,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>204966.84</v>
+        <v>193687.8</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -5046,7 +5046,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>714913.6800000001</v>
+        <v>669244.3199999999</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>1110166.44</v>
+        <v>1049075.76</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -5066,7 +5066,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>395252.76</v>
+        <v>379831.44</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -5159,17 +5159,17 @@
         </is>
       </c>
       <c r="B19" s="36" t="n">
-        <v>337.35</v>
+        <v>335.6</v>
       </c>
       <c r="C19" s="36" t="n">
         <v>429.61</v>
       </c>
       <c r="D19" s="36" t="n">
-        <v>92.26000000000001</v>
+        <v>94.01000000000001</v>
       </c>
       <c r="E19" s="42" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>21.9%</t>
         </is>
       </c>
       <c r="F19" s="49" t="inlineStr">
@@ -5190,17 +5190,17 @@
         </is>
       </c>
       <c r="B20" s="34" t="n">
-        <v>5446.44</v>
+        <v>4280.16</v>
       </c>
       <c r="C20" s="34" t="n">
-        <v>8445.18</v>
+        <v>7505.26</v>
       </c>
       <c r="D20" s="34" t="n">
-        <v>2998.74</v>
+        <v>3225.1</v>
       </c>
       <c r="E20" s="43" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>43.0%</t>
         </is>
       </c>
       <c r="F20" s="49" t="inlineStr">
@@ -5252,17 +5252,17 @@
         </is>
       </c>
       <c r="B22" s="34" t="n">
-        <v>3916.28</v>
+        <v>4307.91</v>
       </c>
       <c r="C22" s="34" t="n">
         <v>7030.58</v>
       </c>
       <c r="D22" s="34" t="n">
-        <v>3114.3</v>
+        <v>2722.67</v>
       </c>
       <c r="E22" s="43" t="inlineStr">
         <is>
-          <t>44.3%</t>
+          <t>38.7%</t>
         </is>
       </c>
       <c r="F22" s="49" t="inlineStr">
@@ -5283,22 +5283,22 @@
         </is>
       </c>
       <c r="B23" s="36" t="n">
-        <v>737.5</v>
+        <v>811.25</v>
       </c>
       <c r="C23" s="36" t="n">
         <v>737.5</v>
       </c>
       <c r="D23" s="36" t="n">
-        <v>0</v>
+        <v>73.75</v>
       </c>
       <c r="E23" s="42" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="F23" s="49" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>GCP</t>
         </is>
       </c>
       <c r="G23" s="51" t="inlineStr">
@@ -5389,22 +5389,22 @@
         </is>
       </c>
       <c r="B28" s="52" t="n">
-        <v>12867.71</v>
+        <v>12045.71</v>
       </c>
       <c r="C28" s="34" t="n">
-        <v>19981.85</v>
+        <v>18882.28</v>
       </c>
       <c r="D28" s="34" t="n">
-        <v>154412.52</v>
+        <v>144548.52</v>
       </c>
       <c r="E28" s="34" t="n">
-        <v>239782.2</v>
+        <v>226587.36</v>
       </c>
       <c r="F28" s="34" t="n">
-        <v>714913.6800000001</v>
+        <v>669244.3199999999</v>
       </c>
       <c r="G28" s="34" t="n">
-        <v>1110166.44</v>
+        <v>1049075.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>